<commit_message>
Fix Excel diagram and detail table spacing
</commit_message>
<xml_diff>
--- a/20261017_144332_A3_IOF_KeepAlive_ACK/A3_Process_IOF_ACK_시나리오_통합평가.xlsx
+++ b/20261017_144332_A3_IOF_KeepAlive_ACK/A3_Process_IOF_ACK_시나리오_통합평가.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet name="DoReady 시나리오" sheetId="1" r:id="R3cfe78bb57804c15"/>
-    <x:sheet name="Process 시나리오" sheetId="3" r:id="R15a1242a09534721"/>
-    <x:sheet name="평가 체크리스트" sheetId="2" r:id="R58f2395f6d104924"/>
+    <x:sheet name="DoReady 시나리오" sheetId="1" r:id="R35d7de4d2fec4bb1"/>
+    <x:sheet name="Process 시나리오" sheetId="3" r:id="R0eff1b66eea94b4b"/>
+    <x:sheet name="평가 체크리스트" sheetId="2" r:id="Rfa61d7bb89fb4036"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10507,7 +10507,7 @@
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="46" t="str">
-        <x:v>수정 가능한 Stage–Process–Vision 객체. 상세177행 / IOF LINE 반복188행 / 1900공통203행 / 완료조건211행. 모든 탭 틀고정 없음.</x:v>
+        <x:v>수정 가능한 Stage–Process–Vision 객체. 상세185행 / IOF LINE 반복196행 / 1900공통211행 / 완료조건219행. 모든 탭 틀고정 없음.</x:v>
       </x:c>
       <x:c r="B6" s="6"/>
       <x:c r="C6" s="6"/>
@@ -11875,610 +11875,548 @@
       <x:c r="E176" s="114"/>
       <x:c r="F176" s="114"/>
     </x:row>
-    <x:row r="177" ht="32" customHeight="1">
-      <x:c r="A177" s="119" t="str">
+    <x:row r="177" ht="20" customHeight="1">
+      <x:c r="A177" s="114"/>
+      <x:c r="B177" s="114"/>
+      <x:c r="C177" s="114"/>
+      <x:c r="D177" s="114"/>
+      <x:c r="E177" s="114"/>
+      <x:c r="F177" s="114"/>
+    </x:row>
+    <x:row r="178" ht="20" customHeight="1">
+      <x:c r="A178" s="114"/>
+      <x:c r="B178" s="114"/>
+      <x:c r="C178" s="114"/>
+      <x:c r="D178" s="114"/>
+      <x:c r="E178" s="114"/>
+      <x:c r="F178" s="114"/>
+    </x:row>
+    <x:row r="179" ht="20" customHeight="1">
+      <x:c r="A179" s="114"/>
+      <x:c r="B179" s="114"/>
+      <x:c r="C179" s="114"/>
+      <x:c r="D179" s="114"/>
+      <x:c r="E179" s="114"/>
+      <x:c r="F179" s="114"/>
+    </x:row>
+    <x:row r="180" ht="20" customHeight="1">
+      <x:c r="A180" s="114"/>
+      <x:c r="B180" s="114"/>
+      <x:c r="C180" s="114"/>
+      <x:c r="D180" s="114"/>
+      <x:c r="E180" s="114"/>
+      <x:c r="F180" s="114"/>
+    </x:row>
+    <x:row r="181" ht="20" customHeight="1">
+      <x:c r="A181" s="114"/>
+      <x:c r="B181" s="114"/>
+      <x:c r="C181" s="114"/>
+      <x:c r="D181" s="114"/>
+      <x:c r="E181" s="114"/>
+      <x:c r="F181" s="114"/>
+    </x:row>
+    <x:row r="182" ht="20" customHeight="1">
+      <x:c r="A182" s="114"/>
+      <x:c r="B182" s="114"/>
+      <x:c r="C182" s="114"/>
+      <x:c r="D182" s="114"/>
+      <x:c r="E182" s="114"/>
+      <x:c r="F182" s="114"/>
+    </x:row>
+    <x:row r="183" ht="20" customHeight="1">
+      <x:c r="A183" s="114"/>
+      <x:c r="B183" s="114"/>
+      <x:c r="C183" s="114"/>
+      <x:c r="D183" s="114"/>
+      <x:c r="E183" s="114"/>
+      <x:c r="F183" s="114"/>
+    </x:row>
+    <x:row r="184" ht="20" customHeight="1">
+      <x:c r="A184" s="114"/>
+      <x:c r="B184" s="114"/>
+      <x:c r="C184" s="114"/>
+      <x:c r="D184" s="114"/>
+      <x:c r="E184" s="114"/>
+      <x:c r="F184" s="114"/>
+    </x:row>
+    <x:row r="185" ht="32" customHeight="1">
+      <x:c r="A185" s="119" t="str">
         <x:v>단계</x:v>
       </x:c>
-      <x:c r="B177" s="120" t="str">
+      <x:c r="B185" s="120" t="str">
         <x:v>시작 신호 / 조건</x:v>
       </x:c>
-      <x:c r="C177" s="120" t="str">
+      <x:c r="C185" s="120" t="str">
         <x:v>Stage PC 동작</x:v>
       </x:c>
-      <x:c r="D177" s="120" t="str">
+      <x:c r="D185" s="120" t="str">
         <x:v>가공 SW 동작·데이터 업데이트</x:v>
       </x:c>
-      <x:c r="E177" s="120" t="str">
+      <x:c r="E185" s="120" t="str">
         <x:v>Vision PC 동작</x:v>
       </x:c>
-      <x:c r="F177" s="121" t="str">
+      <x:c r="F185" s="121" t="str">
         <x:v>완료 기준 / 다음 단계</x:v>
       </x:c>
     </x:row>
-    <x:row r="178" ht="80" customHeight="1">
-      <x:c r="A178" s="20" t="n">
+    <x:row r="186" ht="80" customHeight="1">
+      <x:c r="A186" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B178" s="17" t="str">
+      <x:c r="B186" s="17" t="str">
         <x:v>Stg Process ABLE ON
 Melsec C10A</x:v>
       </x:c>
-      <x:c r="C178" s="122" t="str">
+      <x:c r="C186" s="122" t="str">
         <x:v>Process 진행을 요청하며 Stg Process ABLE을 ON한다.</x:v>
       </x:c>
-      <x:c r="D178" s="17" t="str">
+      <x:c r="D186" s="17" t="str">
         <x:v>DoReady 8단계 전체 완료 전이면 접수를 보류하고 남은 실행 준비를 끝낸다.</x:v>
       </x:c>
-      <x:c r="E178" s="17" t="str">
+      <x:c r="E186" s="17" t="str">
         <x:v>아직 LINE 측정 업무를 시작하지 않는다.</x:v>
       </x:c>
-      <x:c r="F178" s="17" t="str">
+      <x:c r="F186" s="17" t="str">
         <x:v>DoReady8 전체 완료와 Stg Process ABLE 확인 후 2단계.</x:v>
       </x:c>
     </x:row>
-    <x:row r="179" ht="190" customHeight="1">
-      <x:c r="A179" s="20" t="n">
+    <x:row r="187" ht="190" customHeight="1">
+      <x:c r="A187" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B179" s="17" t="str">
+      <x:c r="B187" s="17" t="str">
         <x:v>Process ABLE 조건 성립
 + Process Ready 실제 위치 도착 확인</x:v>
       </x:c>
-      <x:c r="C179" s="122" t="str">
+      <x:c r="C187" s="122" t="str">
         <x:v>0선 옵션을 먼저 확인한다.
 ON: Process Ready 위치 도착을 확인한 현재 PEG 위치 정보를 Melsec에서 받아 ACS에 반영한다.
 OFF: 0선 N·좌표를 읽거나 ACS에 적용하지 않으며 이전 기판의 0선 Trigger를 사용하지 않는다.</x:v>
       </x:c>
-      <x:c r="D179" s="17" t="str">
+      <x:c r="D187" s="17" t="str">
         <x:v>Process Ready 위치 도착·정지 확인 후 Melsec에 PEG 위치 쓰기.
 현재 Glass / Recipe / 0선 옵션과 IOF 측정 LINE 계획을 유지한다.
 Prc Process ABLE을 ON한다. (8208)</x:v>
       </x:c>
-      <x:c r="E179" s="17" t="str">
+      <x:c r="E187" s="17" t="str">
         <x:v>이 단계에서 LINE 측정 업무를 먼저 진행하지 않는다.</x:v>
       </x:c>
-      <x:c r="F179" s="17" t="str">
+      <x:c r="F187" s="17" t="str">
         <x:v>PEG 정보는 이동 중 Melsec 쓰기 금지다. 도착 확인 위치는 Process Ready다. 위치 수치·도착 피드백·실제 주소는 설비 설정과 대조한다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="180" ht="70" customHeight="1">
-      <x:c r="A180" s="20" t="n">
+    <x:row r="188" ht="70" customHeight="1">
+      <x:c r="A188" s="20" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B180" s="17" t="str">
+      <x:c r="B188" s="17" t="str">
         <x:v>Prc Process ABLE ON 확인</x:v>
       </x:c>
-      <x:c r="C180" s="122" t="str">
+      <x:c r="C188" s="122" t="str">
         <x:v>Stg Process START를 ON한다. (C10C)</x:v>
       </x:c>
-      <x:c r="D180" s="17" t="str">
+      <x:c r="D188" s="17" t="str">
         <x:v>Stg Process START를 확인한다.</x:v>
       </x:c>
-      <x:c r="E180" s="17" t="str">
+      <x:c r="E188" s="17" t="str">
         <x:v>준비된 측정 계획을 유지한다.</x:v>
       </x:c>
-      <x:c r="F180" s="17" t="str">
+      <x:c r="F188" s="17" t="str">
         <x:v>Stg START 확인 후 4단계.</x:v>
       </x:c>
     </x:row>
-    <x:row r="181" ht="135" customHeight="1">
-      <x:c r="A181" s="20" t="n">
+    <x:row r="189" ht="135" customHeight="1">
+      <x:c r="A189" s="20" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B181" s="17" t="str">
+      <x:c r="B189" s="17" t="str">
         <x:v>Stg Process START ON 확인</x:v>
       </x:c>
-      <x:c r="C181" s="122" t="str">
+      <x:c r="C189" s="122" t="str">
         <x:v>Prc START 확인 후 역물류 Y 가공 주행을 진행한다.</x:v>
       </x:c>
-      <x:c r="D181" s="17" t="str">
+      <x:c r="D189" s="17" t="str">
         <x:v>Prc Process START를 ON한다. (820A)
 Glass / Recipe / LINE i / Frame k / 요청 UID 문맥을 관리한다. 이미 실행한 Zero Set·A1/8 Task를 다시 실행하지 않는다.</x:v>
       </x:c>
-      <x:c r="E181" s="17" t="str">
+      <x:c r="E189" s="17" t="str">
         <x:v>LINE별 준비·촬영·결과 문맥을 구분한다.</x:v>
       </x:c>
-      <x:c r="F181" s="17" t="str">
+      <x:c r="F189" s="17" t="str">
         <x:v>START 신호와 실제 첫 출사를 구분한다. 실제 MOF 가공이 먼저 시작되고 Review Camera가 뒤따라 촬영한다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="182" ht="225" customHeight="1">
-      <x:c r="A182" s="20" t="n">
+    <x:row r="190" ht="225" customHeight="1">
+      <x:c r="A190" s="20" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B182" s="17" t="str">
+      <x:c r="B190" s="17" t="str">
         <x:v>실제 MOF 가공 시작
 0선 IOF를 별도로 병행</x:v>
       </x:c>
-      <x:c r="C182" s="122" t="str">
+      <x:c r="C190" s="122" t="str">
         <x:v>가공 Y는 연속 주행한다. 각 LINE 촬영 중 Review X를 유지한다.
 현재 측정의1002 ACK를 Process가 수신한 뒤 다음 Review X 이동 요청을 받아 이동한다.</x:v>
       </x:c>
-      <x:c r="D182" s="123" t="str">
+      <x:c r="D190" s="123" t="str">
         <x:v>0선 ON: 측정 i=1~N마다 시퀀스 시작 때1900을1회 확인한다. 정상 응답 후1001 Ready ACK → LINE 연속 촬영 → LINE 끝·마지막 노출 종료 →1002 ACK 수신 →1003 결과를 진행한다.
 1002 ACK 수신 시 다음 Review X(i+1) Melsec 요청을 시작하고1003 처리와 병행한다.1002/1003 앞에1900을 다시 호출하지 않는다.
 0선 OFF는 이 분기를 생략한다.</x:v>
       </x:c>
-      <x:c r="E182" s="123" t="str">
+      <x:c r="E190" s="123" t="str">
         <x:v>각 측정 시퀀스 시작의1900에 응답하고1001로 해당 LINE을 준비한다. Trigger별 Grab·검사를 진행하고1002 ACK 후1003 결과를 계약대로 회신한다.</x:v>
       </x:c>
-      <x:c r="F182" s="123" t="str">
+      <x:c r="F190" s="123" t="str">
         <x:v>정상 N회 측정의1900 요청은 총 N회다.1002 ACK는 검사 전체 완료와 다르며, 다음 X 요청은 이 ACK를 Process가 받은 뒤에만 시작한다.1003 송신·결과는 X 이동의 선행조건이 아니다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="183" ht="200" customHeight="1">
-      <x:c r="A183" s="20" t="n">
+    <x:row r="191" ht="200" customHeight="1">
+      <x:c r="A191" s="20" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B183" s="17" t="str">
+      <x:c r="B191" s="17" t="str">
         <x:v>가공·0선 시퀀스 완료 합류</x:v>
       </x:c>
-      <x:c r="C183" s="122" t="str">
+      <x:c r="C191" s="122" t="str">
         <x:v>가공이 먼저 끝나도 마지막 필요한 LINE 촬영까지 유한 Y 주행을 유지한다. 마지막 노출과 계획된 감속·정지 후 TCP만 남았다면 정지 상태에서 처리할 수 있다.</x:v>
       </x:c>
-      <x:c r="D183" s="123" t="str">
+      <x:c r="D191" s="123" t="str">
         <x:v>실제 출사 종료는 MachiningDone으로 보존한다.
 0선 ON: MachiningDone AND ZeroSequenceDone일 때만 Prc Process COMPLETE를 ON한다. (820C)
 0선 OFF: MachiningDone으로 완료한다.
 0선Done은 필요한 모든 LINE의 실제 촬영과 결과 처리/시퀀스 종결 완료다.</x:v>
       </x:c>
-      <x:c r="E183" s="123" t="str">
+      <x:c r="E191" s="123" t="str">
         <x:v>가공 종료 후에도 잔여 촬영·검사·LINE 결과 처리를 계속한다.</x:v>
       </x:c>
-      <x:c r="F183" s="123" t="str">
+      <x:c r="F191" s="123" t="str">
         <x:v>어느 분기가 먼저 끝나도 합류 전 상위 COMPLETE는 OFF다. LINE 끝·가공Done·Y 주행Done·0선Done은 서로 구분한다. NG와 미촬영/미수신도 구분한다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="184" ht="125" customHeight="1">
-      <x:c r="A184" s="20" t="n">
+    <x:row r="192" ht="125" customHeight="1">
+      <x:c r="A192" s="20" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B184" s="17" t="str">
+      <x:c r="B192" s="17" t="str">
         <x:v>Prc Process COMPLETE ON 확인</x:v>
       </x:c>
-      <x:c r="C184" s="122" t="str">
+      <x:c r="C192" s="122" t="str">
         <x:v>Prc COMPLETE와 계획된 실제 Y 주행 종료를 확인한 뒤 Stg Process COMPLETE를 ON한다. (C10E)</x:v>
       </x:c>
-      <x:c r="D184" s="17" t="str">
+      <x:c r="D192" s="17" t="str">
         <x:v>Stg Process COMPLETE를 확인한다. 합류 전에 All OFF·다음 기판 제어권 이관을 하지 않는다.</x:v>
       </x:c>
-      <x:c r="E184" s="17" t="str">
+      <x:c r="E192" s="17" t="str">
         <x:v>현재 기판의 필요한 결과와 잔여 거래를 확인한다.</x:v>
       </x:c>
-      <x:c r="F184" s="17" t="str">
+      <x:c r="F192" s="17" t="str">
         <x:v>Prc COMPLETE → Stg COMPLETE 순서를 유지한다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="185" ht="145" customHeight="1">
-      <x:c r="A185" s="20" t="n">
+    <x:row r="193" ht="145" customHeight="1">
+      <x:c r="A193" s="20" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B185" s="17" t="str">
+      <x:c r="B193" s="17" t="str">
         <x:v>Stg Process COMPLETE ON 확인</x:v>
       </x:c>
-      <x:c r="C185" s="122" t="str">
+      <x:c r="C193" s="122" t="str">
         <x:v>ReviewDone과 X 이동 허가 확인 후 다음 기판 선배치를 진행한다.</x:v>
       </x:c>
-      <x:c r="D185" s="17" t="str">
+      <x:c r="D193" s="17" t="str">
         <x:v>현재 기판의 가공·LINE별 결과/NG/미완료를 화면·이력에 정리한다. Prc All OFF → Stg All OFF 복귀와 합의한 후속 조건을 처리한다.</x:v>
       </x:c>
-      <x:c r="E185" s="17" t="str">
+      <x:c r="E193" s="17" t="str">
         <x:v>늦은 응답은 원래 Glass / LINE / Frame 문맥에만 연결한다.</x:v>
       </x:c>
-      <x:c r="F185" s="17" t="str">
+      <x:c r="F193" s="17" t="str">
         <x:v>미수신을 OK/해당없음으로 바꾸지 않는다. 오류 종결의 정상 COMPLETE 허용과 후속 조건은 계약으로 확정한다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="186" ht="24" customHeight="1">
-      <x:c r="A186" s="3"/>
-      <x:c r="B186" s="3"/>
-      <x:c r="C186" s="3"/>
-      <x:c r="D186" s="3"/>
-      <x:c r="E186" s="3"/>
-      <x:c r="F186" s="3"/>
-    </x:row>
-    <x:row r="187" ht="24" customHeight="1">
-      <x:c r="A187" s="3"/>
-      <x:c r="B187" s="3"/>
-      <x:c r="C187" s="3"/>
-      <x:c r="D187" s="3"/>
-      <x:c r="E187" s="3"/>
-      <x:c r="F187" s="3"/>
-    </x:row>
-    <x:row r="188" ht="32" customHeight="1">
-      <x:c r="A188" s="119" t="str">
+    <x:row r="194" ht="24" customHeight="1">
+      <x:c r="A194" s="3"/>
+      <x:c r="B194" s="3"/>
+      <x:c r="C194" s="3"/>
+      <x:c r="D194" s="3"/>
+      <x:c r="E194" s="3"/>
+      <x:c r="F194" s="3"/>
+    </x:row>
+    <x:row r="195" ht="24" customHeight="1">
+      <x:c r="A195" s="3"/>
+      <x:c r="B195" s="3"/>
+      <x:c r="C195" s="3"/>
+      <x:c r="D195" s="3"/>
+      <x:c r="E195" s="3"/>
+      <x:c r="F195" s="3"/>
+    </x:row>
+    <x:row r="196" ht="32" customHeight="1">
+      <x:c r="A196" s="119" t="str">
         <x:v>단계</x:v>
       </x:c>
-      <x:c r="B188" s="120" t="str">
+      <x:c r="B196" s="120" t="str">
         <x:v>시작 신호 / 조건</x:v>
       </x:c>
-      <x:c r="C188" s="120" t="str">
+      <x:c r="C196" s="120" t="str">
         <x:v>Stage PC 동작</x:v>
       </x:c>
-      <x:c r="D188" s="120" t="str">
+      <x:c r="D196" s="120" t="str">
         <x:v>가공 SW 동작·데이터 업데이트</x:v>
       </x:c>
-      <x:c r="E188" s="120" t="str">
+      <x:c r="E196" s="120" t="str">
         <x:v>Vision PC 동작</x:v>
       </x:c>
-      <x:c r="F188" s="121" t="str">
+      <x:c r="F196" s="121" t="str">
         <x:v>완료 기준 / 다음 단계</x:v>
       </x:c>
     </x:row>
-    <x:row r="189" ht="145" customHeight="1">
-      <x:c r="A189" s="20" t="str">
+    <x:row r="197" ht="145" customHeight="1">
+      <x:c r="A197" s="20" t="str">
         <x:v>5-1</x:v>
       </x:c>
-      <x:c r="B189" s="17" t="str">
+      <x:c r="B197" s="17" t="str">
         <x:v>0선 ON / IOF LINE 계획 선택</x:v>
       </x:c>
-      <x:c r="C189" s="122" t="str">
+      <x:c r="C197" s="122" t="str">
         <x:v>Y 가공 주행을 계속하며 현재 LINE i의 Review X 이동을 준비한다.</x:v>
       </x:c>
-      <x:c r="D189" s="123" t="str">
+      <x:c r="D197" s="123" t="str">
         <x:v>측정 i=1~N의 각 IOF 시퀀스와 LINE 안 Frame k를 구분한다. 현재 Glass / Recipe / i / 대상 배열·촬영 구간을 보존한다. 각 i 시작 때1900을1회 확인하며 이전 시퀀스의 성공을 다음 i에 재사용하지 않는다.</x:v>
       </x:c>
-      <x:c r="E189" s="123" t="str">
+      <x:c r="E197" s="123" t="str">
         <x:v>현재 LINE과 이전 LINE의 준비/이미지/결과 문맥을 구분한다.</x:v>
       </x:c>
-      <x:c r="F189" s="123" t="str">
+      <x:c r="F197" s="123" t="str">
         <x:v>N은 IOF 측정 시퀀스 수이며 정상 N회면1900 총 N번이다. nHoleCnt·Trigger/Frame/Mark 수와 구분한다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="190" ht="160" customHeight="1">
-      <x:c r="A190" s="20" t="str">
+    <x:row r="198" ht="160" customHeight="1">
+      <x:c r="A198" s="20" t="str">
         <x:v>5-2</x:v>
       </x:c>
-      <x:c r="B190" s="17" t="str">
+      <x:c r="B198" s="17" t="str">
         <x:v>현재 LINE 시작 위치 준비</x:v>
       </x:c>
-      <x:c r="C190" s="122" t="str">
+      <x:c r="C198" s="122" t="str">
         <x:v>현재 또는 미리 요청받은 Review X를 이동·정착시킨다. Y 연속 주행을 유지한다.</x:v>
       </x:c>
-      <x:c r="D190" s="123" t="str">
+      <x:c r="D198" s="123" t="str">
         <x:v>X 허가·이전 요청 복귀 확인 후8011 목표X·8015 속도·801B 모드를 기록하고8029 Request ON. C128 후보와 현재 요청의 실제 도착·정착을 대조한 뒤 Request OFF/복귀를 확인한다.</x:v>
       </x:c>
-      <x:c r="E190" s="123" t="str">
+      <x:c r="E198" s="123" t="str">
         <x:v>현재 LINE 결과를 다음 준비로 덮어쓰지 않는다.</x:v>
       </x:c>
-      <x:c r="F190" s="123" t="str">
+      <x:c r="F198" s="123" t="str">
         <x:v>첫 X는 첫 측정 시작 전에 준비한다. 다음 X(i+1)는 현재 i의1002 정상 ACK 수신 후 시작한다. X 도착과 Trigger/Grab은 별도 상태다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="191" ht="175" customHeight="1">
-      <x:c r="A191" s="20" t="str">
+    <x:row r="199" ht="175" customHeight="1">
+      <x:c r="A199" s="20" t="str">
         <x:v>5-3</x:v>
       </x:c>
-      <x:c r="B191" s="17" t="str">
+      <x:c r="B199" s="17" t="str">
         <x:v>LINE i 시작 위치 도착 확인
 현재 LINE 업무 시작</x:v>
       </x:c>
-      <x:c r="C191" s="122" t="str">
+      <x:c r="C199" s="122" t="str">
         <x:v>Review X 도착·정착과 LINE 시작 구간 조건을 확인한다. 이를 위해 진행 중 Y를 점마다 정지하지 않는다.</x:v>
       </x:c>
-      <x:c r="D191" s="124" t="str">
+      <x:c r="D199" s="124" t="str">
         <x:v>측정 i 시퀀스 시작에서1900을1회 보내고 정상 응답을 확인한다. 이어1001 FlyingReady와 업무 UID의 정상 ACK를 확인한다. nType은 IOF로 설정하고 해당 LINE의 nHoleCnt·stMarkSearch[]를 보낸다.1002·1003 앞에서1900을 재호출하지 않는다.</x:v>
       </x:c>
-      <x:c r="E191" s="124" t="str">
+      <x:c r="E199" s="124" t="str">
         <x:v>해당 LINE의 IOF/TRG Mode·조명·노출·대상 배열을 준비한 뒤 FlyingReady ACK를 보낸다.</x:v>
       </x:c>
-      <x:c r="F191" s="124" t="str">
+      <x:c r="F199" s="124" t="str">
         <x:v>정상 N회 시퀀스면1900 N회다. 다음 i는 현재 결과 확인 뒤 새로운 초기1900·1001을 진행한다.1900 확인 성공 범위는 현재 i/연결 문맥이며 첫 Trigger 전에 Ready ACK를 확보한다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="192" ht="170" customHeight="1">
-      <x:c r="A192" s="20" t="str">
+    <x:row r="200" ht="170" customHeight="1">
+      <x:c r="A200" s="20" t="str">
         <x:v>5-4</x:v>
       </x:c>
-      <x:c r="B192" s="17" t="str">
+      <x:c r="B200" s="17" t="str">
         <x:v>1001 Ready ACK 후
 LINE i의 IOF 촬영 구간</x:v>
       </x:c>
-      <x:c r="C192" s="122" t="str">
+      <x:c r="C200" s="122" t="str">
         <x:v>연속 Y가 LINE의 PEG Trigger 위치들을 통과할 때 HW Trigger를 발생시킨다. 촬영 중 Review X를 유지한다.</x:v>
       </x:c>
-      <x:c r="D192" s="123" t="str">
+      <x:c r="D200" s="123" t="str">
         <x:v>실제 TriggerObserved[i,k]와 Frame·대상 대응을 기록한다. LINE 시작→끝 구간의 실제 Trigger를 추적한다. X 도착/예약시각을 실제 Trigger로 대체하지 않는다.</x:v>
       </x:c>
-      <x:c r="E192" s="123" t="str">
+      <x:c r="E200" s="123" t="str">
         <x:v>각 HW Trigger 순간 Grab → 노출·취득·검사. LINE 안 여러 Trigger/Frame을 원래 대상 순서로 유지한다.</x:v>
       </x:c>
-      <x:c r="F192" s="123" t="str">
+      <x:c r="F200" s="123" t="str">
         <x:v>첫/중간 Grab마다 다음 X로 이동하거나1002/1003을 보내 LINE을 끝내지 않는다. 촬영 수·배열 대응은 실제 계획과 대조한다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="193" ht="175" customHeight="1">
-      <x:c r="A193" s="20" t="str">
+    <x:row r="201" ht="175" customHeight="1">
+      <x:c r="A201" s="20" t="str">
         <x:v>5-5</x:v>
       </x:c>
-      <x:c r="B193" s="17" t="str">
+      <x:c r="B201" s="17" t="str">
         <x:v>LINE 끝 구간 도달
 마지막 유효 Trigger·노출 종료</x:v>
       </x:c>
-      <x:c r="C193" s="122" t="str">
+      <x:c r="C201" s="122" t="str">
         <x:v>현재 LINE 끝과 마지막 노출 종료를 확인하며 Y는 계속 주행한다. 아직1002 ACK를 Process가 받기 전에는 다음 Review X 요청을 시작하지 않는다.</x:v>
       </x:c>
-      <x:c r="D193" s="123" t="str">
+      <x:c r="D201" s="123" t="str">
         <x:v>LINE 끝·필요한 Trigger/Frame·마지막 노출 종료를 확인하고1002를 송신한다. 현재 i의 정상1002 ACK 수신 여부를 기다린다. 이 구간에는 추가1900과 다음 X 요청을 넣지 않는다.</x:v>
       </x:c>
-      <x:c r="E193" s="123" t="str">
+      <x:c r="E201" s="123" t="str">
         <x:v>현재 LINE 검사/결과 문맥을 유지한다. 다음 X 선배치와 다음 LINE1001 준비를 구분한다.</x:v>
       </x:c>
-      <x:c r="F193" s="123" t="str">
+      <x:c r="F201" s="123" t="str">
         <x:v>LINE 끝은 Y 정지가 아니다. 다음 X는 정상1002 ACK 수신이 필요하다. i=N이면 다음 측정 X 요청은 생략한다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="194" ht="165" customHeight="1">
-      <x:c r="A194" s="20" t="str">
+    <x:row r="202" ht="165" customHeight="1">
+      <x:c r="A202" s="20" t="str">
         <x:v>5-6</x:v>
       </x:c>
-      <x:c r="B194" s="17" t="str">
+      <x:c r="B202" s="17" t="str">
         <x:v>Vision1002 ACK를
 Process가 정상 수신</x:v>
       </x:c>
-      <x:c r="C194" s="122" t="str">
+      <x:c r="C202" s="122" t="str">
         <x:v>Process의 Melsec 좌표/Request를 받아 다음 Review X를 이동한다. Y 주행은 계속한다.</x:v>
       </x:c>
-      <x:c r="D194" s="124" t="str">
+      <x:c r="D202" s="124" t="str">
         <x:v>Cmd1002·요청 UID·Error·Len 등 정상 ACK를 현재 i 문맥에서 검증한다. 수신 시 다음 이동 대상을 i+1로 고정한다. X 허가·이전 요청 복귀 확인 후8011/8015/801B 기록 →8029 Request로 다음 X 이동을 시작한다.1003 송신/응답은 기다리지 않는다.</x:v>
       </x:c>
-      <x:c r="E194" s="124" t="str">
+      <x:c r="E202" s="124" t="str">
         <x:v>1002 상태 ACK를 회신한다. 해당 LINE 측정/검사를 계속 마무리하며1003의 결과 응답 준비는 별도로 처리한다.</x:v>
       </x:c>
-      <x:c r="F194" s="124" t="str">
+      <x:c r="F202" s="124" t="str">
         <x:v>ACK 지연·누락·오류·UID 불일치 동안 다음 X Request는 없다. 정상 ACK 수신 이후에만 요청한다.1002 ACK를 검사 전체 완료나0선Done으로 대체하지 않는다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="195" ht="165" customHeight="1">
-      <x:c r="A195" s="20" t="str">
+    <x:row r="203" ht="165" customHeight="1">
+      <x:c r="A203" s="20" t="str">
         <x:v>5-7</x:v>
       </x:c>
-      <x:c r="B195" s="17" t="str">
+      <x:c r="B203" s="17" t="str">
         <x:v>1002 정상 ACK 이후
 다음 X 이동과1003 병행</x:v>
       </x:c>
-      <x:c r="C195" s="122" t="str">
+      <x:c r="C203" s="122" t="str">
         <x:v>다음 X 이동·정착을1003 결과 요청/검사/응답과 병행한다.1003 지연 때문에 X 시작을 늦추지 않는다.</x:v>
       </x:c>
-      <x:c r="D195" s="124" t="str">
+      <x:c r="D203" s="124" t="str">
         <x:v>현재 i의 측정 완료/1003 응답 준비 계약에 따라1003 MarkFindLine 결과를 요청·처리한다. 추가1900을 넣지 않는다. 다음 X 이동 대상 i+1과 현재 결과 대상 i를 분리하며 두 경로를 서로 기다리게 하지 않는다.</x:v>
       </x:c>
-      <x:c r="E195" s="124" t="str">
+      <x:c r="E203" s="124" t="str">
         <x:v>해당 LINE 측정 완료 후 계약된1003 결과 범위·순서로 회신한다.</x:v>
       </x:c>
-      <x:c r="F195" s="124" t="str">
+      <x:c r="F203" s="124" t="str">
         <x:v>X 개시 조건은1002 정상 ACK 수신이며1003 송신·응답·결과 완료가 아니다. Vision 측정 완료/응답 준비·Timeout은 기존 계약을 따른다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="196" ht="165" customHeight="1">
-      <x:c r="A196" s="20" t="str">
+    <x:row r="204" ht="165" customHeight="1">
+      <x:c r="A204" s="20" t="str">
         <x:v>5-8</x:v>
       </x:c>
-      <x:c r="B196" s="17" t="str">
+      <x:c r="B204" s="17" t="str">
         <x:v>현재 LINE1003 결과 수신</x:v>
       </x:c>
-      <x:c r="C196" s="122" t="str">
+      <x:c r="C204" s="122" t="str">
         <x:v>다음 LINE XReady를 보존한다. 결과가 도착할 때까지 X 이동 자체를 늦추지 않는다.</x:v>
       </x:c>
-      <x:c r="D196" s="123" t="str">
+      <x:c r="D204" s="123" t="str">
         <x:v>Cmd·업무 UID·Error·Len·개수·순서를 검증하고 원래 Glass / LINE i / Frame·슬롯에 nResult·TargetMark/Hole pixel을 저장한다. Table·화면·이력을 갱신한다.</x:v>
       </x:c>
-      <x:c r="E196" s="123" t="str">
+      <x:c r="E204" s="123" t="str">
         <x:v>실패 슬롯을 유지하고 현재 LINE의 계약된 결과를 회신한다.</x:v>
       </x:c>
-      <x:c r="F196" s="123" t="str">
+      <x:c r="F204" s="123" t="str">
         <x:v>1002/1003 Body의 LINE 식별자가 있다고 가정하지 않는다. 요청 UID와 내부 원래 LINE/배열 문맥으로 대응하며 현재 이동 대상에 결과를 넣지 않는다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="197" ht="185" customHeight="1">
-      <x:c r="A197" s="20" t="str">
+    <x:row r="205" ht="185" customHeight="1">
+      <x:c r="A205" s="20" t="str">
         <x:v>5-9</x:v>
       </x:c>
-      <x:c r="B197" s="17" t="str">
+      <x:c r="B205" s="17" t="str">
         <x:v>현재 LINE 결과 확인 후
 다음 LINE 반복</x:v>
       </x:c>
-      <x:c r="C197" s="122" t="str">
+      <x:c r="C205" s="122" t="str">
         <x:v>이미 선배치한 다음 Review X의 실제 도착·정착을 확인한다. 다음 LINE 첫 촬영 전까지 준비 시간을 확보한다.</x:v>
       </x:c>
-      <x:c r="D197" s="123" t="str">
+      <x:c r="D205" s="123" t="str">
         <x:v>현재 결과 확인 후 i+1로 시퀀스 문맥을 전환한다. 이미 요청한 다음 XReady와 시작 구간을 확인하고 새로운 시퀀스 초기1900 1회 →1001/ACK → 촬영을 반복한다.</x:v>
       </x:c>
-      <x:c r="E197" s="123" t="str">
+      <x:c r="E205" s="123" t="str">
         <x:v>이전 LINE 결과 확인 후 다음1001로 준비 문맥을 갱신한다.</x:v>
       </x:c>
-      <x:c r="F197" s="123" t="str">
+      <x:c r="F205" s="123" t="str">
         <x:v>다음 촬영 마감에는 LINE 종료→1002 ACK 지연→X 요청·이동·정착 시간을 포함한다.1003 결과·다음 초기1900/1001 준비 경로도 별도로 평가한다. 미준비/초과는 미완료이며 현재 Y 정지·역주행·이동 중 PEG 재기록으로 만회하지 않는다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="198" ht="170" customHeight="1">
-      <x:c r="A198" s="20" t="str">
+    <x:row r="206" ht="170" customHeight="1">
+      <x:c r="A206" s="20" t="str">
         <x:v>5-10</x:v>
       </x:c>
-      <x:c r="B198" s="17" t="str">
+      <x:c r="B206" s="17" t="str">
         <x:v>MachiningDone 선행
 0선 LINE 잔여 있음</x:v>
       </x:c>
-      <x:c r="C198" s="122" t="str">
+      <x:c r="C206" s="122" t="str">
         <x:v>마지막 필요한 LINE의 Trigger·노출까지 유한 Y 주행을 계속하고 계획된 감속/정지를 마친다.</x:v>
       </x:c>
-      <x:c r="D198" s="123" t="str">
+      <x:c r="D206" s="123" t="str">
         <x:v>가공Done만 보존하고 상위 COMPLETE는 OFF다. 잔여 X·LINE별1001·Trigger/Grab·1002·측정 완료·1003 결과를 계속 처리한다.</x:v>
       </x:c>
-      <x:c r="E198" s="123" t="str">
+      <x:c r="E206" s="123" t="str">
         <x:v>남은 LINE의 촬영·검사·결과를 처리한다.</x:v>
       </x:c>
-      <x:c r="F198" s="123" t="str">
+      <x:c r="F206" s="123" t="str">
         <x:v>촬영이 끝나고 TCP만 남았으면 Y 정지 상태에서 처리할 수 있다. 가공Done으로 잔여 촬영을 종료하지 않는다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="199" ht="170" customHeight="1">
-      <x:c r="A199" s="20" t="str">
+    <x:row r="207" ht="170" customHeight="1">
+      <x:c r="A207" s="20" t="str">
         <x:v>5-11</x:v>
       </x:c>
-      <x:c r="B199" s="17" t="str">
+      <x:c r="B207" s="17" t="str">
         <x:v>0선Done 선행 또는
 두 시퀀스 완료 합류</x:v>
       </x:c>
-      <x:c r="C199" s="122" t="str">
+      <x:c r="C207" s="122" t="str">
         <x:v>0선 촬영이 먼저 끝나도 현재 가공 주행을 계속한다.</x:v>
       </x:c>
-      <x:c r="D199" s="123" t="str">
+      <x:c r="D207" s="123" t="str">
         <x:v>필요한 모든 LINE의 실제 촬영·결과 처리/시퀀스 종결 완료를0선Done으로 보존한다. ON은 가공Done AND0선Done, OFF는 가공Done으로 상위 완료한다.</x:v>
       </x:c>
-      <x:c r="E199" s="123" t="str">
+      <x:c r="E207" s="123" t="str">
         <x:v>NG 판정과 미촬영/미수신 미완료를 구분한다.</x:v>
       </x:c>
-      <x:c r="F199" s="123" t="str">
+      <x:c r="F207" s="123" t="str">
         <x:v>작업자 종료·Timeout·마지막 Trigger 예약을 정상0선Done으로 바꾸지 않는다. 합류 전 All OFF/제어권 이관을 하지 않는다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="200" ht="180" customHeight="1">
-      <x:c r="A200" s="20" t="str">
+    <x:row r="208" ht="180" customHeight="1">
+      <x:c r="A208" s="20" t="str">
         <x:v>5-12</x:v>
       </x:c>
-      <x:c r="B200" s="17" t="str">
+      <x:c r="B208" s="17" t="str">
         <x:v>일반 측정/TCP 오류
 또는 후행 결과/복구</x:v>
       </x:c>
-      <x:c r="C200" s="122" t="str">
+      <x:c r="C208" s="122" t="str">
         <x:v>현재 MOF를 끝까지 진행한다. 비상정지·안전 인터록은 기존 기준이다.</x:v>
       </x:c>
-      <x:c r="D200" s="123" t="str">
+      <x:c r="D208" s="123" t="str">
         <x:v>시퀀스 초기1900 실패면1001과 해당 후속을 시작하지 않는다. 진행 중 소켓 손실/업무 실패는 현재 i 미완료로 보존한다.1002/1003 앞1900을 자동 재삽입해 정상 재개했다고 간주하지 않는다. 같은 연결 초기1900은 동시1건이며 늦은UID0·실패 세션을 보호한다.</x:v>
       </x:c>
-      <x:c r="E200" s="123" t="str">
+      <x:c r="E208" s="123" t="str">
         <x:v>연결 복구만으로 이전 이미지·검사 결과가 복구됐다고 간주하지 않는다.</x:v>
       </x:c>
-      <x:c r="F200" s="123" t="str">
+      <x:c r="F208" s="123" t="str">
         <x:v>누락을 정상 촬영/OK/0선Done으로 만들지 않는다. 오류 종결·재검·후속 허용은 계약으로 확정한다.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="201" ht="24" customHeight="1">
-      <x:c r="A201" s="3"/>
-      <x:c r="B201" s="3"/>
-      <x:c r="C201" s="3"/>
-      <x:c r="D201" s="3"/>
-      <x:c r="E201" s="3"/>
-      <x:c r="F201" s="3"/>
-    </x:row>
-    <x:row r="202" ht="24" customHeight="1">
-      <x:c r="A202" s="3"/>
-      <x:c r="B202" s="3"/>
-      <x:c r="C202" s="3"/>
-      <x:c r="D202" s="3"/>
-      <x:c r="E202" s="3"/>
-      <x:c r="F202" s="3"/>
-    </x:row>
-    <x:row r="203" ht="32" customHeight="1">
-      <x:c r="A203" s="119" t="str">
-        <x:v>단계</x:v>
-      </x:c>
-      <x:c r="B203" s="120" t="str">
-        <x:v>시작 신호 / 조건</x:v>
-      </x:c>
-      <x:c r="C203" s="120" t="str">
-        <x:v>Stage PC 동작</x:v>
-      </x:c>
-      <x:c r="D203" s="120" t="str">
-        <x:v>가공 SW 동작·데이터 업데이트</x:v>
-      </x:c>
-      <x:c r="E203" s="120" t="str">
-        <x:v>Vision PC 동작</x:v>
-      </x:c>
-      <x:c r="F203" s="121" t="str">
-        <x:v>완료 기준 / 다음 단계</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="204" ht="165" customHeight="1">
-      <x:c r="A204" s="20" t="str">
-        <x:v>공통1</x:v>
-      </x:c>
-      <x:c r="B204" s="17" t="str">
-        <x:v>측정 i 시퀀스 시작
-1900 1회</x:v>
-      </x:c>
-      <x:c r="C204" s="17" t="str">
-        <x:v>Stage Melsec 축 요청과 구분한다.</x:v>
-      </x:c>
-      <x:c r="D204" s="124" t="str">
-        <x:v>각 i=1~N의 IOF 전체 시퀀스 시작에서1900 요청/정상 응답을1회 확인한다. 이후 같은 시퀀스의1001→1002→1003 앞마다 다시 확인하지 않는다. 정상 N회면1900 요청 N회이며0선 OFF는 이 분기를 생략한다.</x:v>
-      </x:c>
-      <x:c r="E204" s="124" t="str">
-        <x:v>1900 요청/응답은 Cmd1900·UID0·Body0·Error0이다.1999는 별도 Heartbeat로 초기1900 응답을 대체하지 않는다.</x:v>
-      </x:c>
-      <x:c r="F204" s="124" t="str">
-        <x:v>성공 범위는 현재 Glass/i/연결 문맥이다. 이전 i의 성공을 다음 i의 초기 확인으로 재사용하지 않는다.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="205" ht="165" customHeight="1">
-      <x:c r="A205" s="20" t="str">
-        <x:v>공통2</x:v>
-      </x:c>
-      <x:c r="B205" s="17" t="str">
-        <x:v>초기1900 오류/불일치/Timeout</x:v>
-      </x:c>
-      <x:c r="C205" s="17" t="str">
-        <x:v>이미 시작한 MOF와 Y 주행은 계속한다.</x:v>
-      </x:c>
-      <x:c r="D205" s="124" t="str">
-        <x:v>해당 i의1001/측정 후속을 시작하지 않고 원인·문맥·미완료를 남긴다.1002/1003 앞 추가1900으로 만회하는 흐름을 만들지 않는다.</x:v>
-      </x:c>
-      <x:c r="E205" s="124" t="str">
-        <x:v>잘못된 Cmd/UID/Len/Error 또는1999를 정상1900으로 취급하지 않는다.</x:v>
-      </x:c>
-      <x:c r="F205" s="124" t="str">
-        <x:v>정상 N회=N번과 오류/재시도 횟수는 구분한다. 복구·재시도 정책 수치는 계약으로 확정한다.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="206" ht="180" customHeight="1">
-      <x:c r="A206" s="20" t="str">
-        <x:v>공통3</x:v>
-      </x:c>
-      <x:c r="B206" s="17" t="str">
-        <x:v>연결 손실·늦은 응답
-새 시퀀스 경계</x:v>
-      </x:c>
-      <x:c r="C206" s="17" t="str">
-        <x:v>1002 ACK 미수신 중에는 다음 X Request를 시작하지 않는다.</x:v>
-      </x:c>
-      <x:c r="D206" s="124" t="str">
-        <x:v>현재 거래·이미지/결과 문맥을 보존하고 연결 복구만으로 현재 시퀀스를 완료 처리하지 않는다. 새로운 시퀀스를 정식 시작하면 그 시작에서1900을1회 확인한다. 실패 세션·UID0 지연 응답 보호와 재동기화는 추가 설계다.</x:v>
-      </x:c>
-      <x:c r="E206" s="124" t="str">
-        <x:v>1002 상태 ACK와 검사 완료·1003 결과를 구분한다. 복구된 연결이 이전 버퍼 복구를 뜻하지 않는다.</x:v>
-      </x:c>
-      <x:c r="F206" s="124" t="str">
-        <x:v>현재 시퀀스 중간에1900을 임의로 재삽입하지 않는다. 재검/새 시퀀스 허용은 계약으로 확인한다.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="207" ht="140" customHeight="1">
-      <x:c r="A207" s="20" t="str">
-        <x:v>공통4</x:v>
-      </x:c>
-      <x:c r="B207" s="17" t="str">
-        <x:v>Process 도식의 화살표·방향 읽기</x:v>
-      </x:c>
-      <x:c r="C207" s="17" t="str">
-        <x:v>남색 실선: Stage↔Process의 Melsec 신호/좌표/축 요청·완료.</x:v>
-      </x:c>
-      <x:c r="D207" s="124" t="str">
-        <x:v>주황 실선: Process→Vision TCP 요청. 초록 실선: Vision→Process TCP 응답/ACK/결과. 수평 화살촉이 수신자다.</x:v>
-      </x:c>
-      <x:c r="E207" s="124" t="str">
-        <x:v>보라 실선: Stage→Vision HW Trigger. Process Trigger 관측은 내부 동작 상자로 표시하고 미정 통신 경로를 만들지 않는다.</x:v>
-      </x:c>
-      <x:c r="F207" s="124" t="str">
-        <x:v>Process 도식의 세로선은 PC별 시간 흐름이며 메시지가 아니다. ACK 이후 X 이동과1003은 병행 경로다. 화살표 높이는 정확한 경과시간이나 양쪽 완료 시각 일치를 뜻하지 않는다.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="208" ht="24" customHeight="1">
-      <x:c r="A208" s="3"/>
-      <x:c r="B208" s="3"/>
-      <x:c r="C208" s="3"/>
-      <x:c r="D208" s="3"/>
-      <x:c r="E208" s="3"/>
-      <x:c r="F208" s="3"/>
     </x:row>
     <x:row r="209" ht="24" customHeight="1">
       <x:c r="A209" s="3"/>
@@ -12498,123 +12436,113 @@
     </x:row>
     <x:row r="211" ht="32" customHeight="1">
       <x:c r="A211" s="119" t="str">
-        <x:v>조건</x:v>
+        <x:v>단계</x:v>
       </x:c>
       <x:c r="B211" s="120" t="str">
-        <x:v>실제 가공 상태</x:v>
+        <x:v>시작 신호 / 조건</x:v>
       </x:c>
       <x:c r="C211" s="120" t="str">
-        <x:v>0선방어 상태</x:v>
+        <x:v>Stage PC 동작</x:v>
       </x:c>
       <x:c r="D211" s="120" t="str">
         <x:v>가공 SW 동작·데이터 업데이트</x:v>
       </x:c>
       <x:c r="E211" s="120" t="str">
-        <x:v>물리 주행 / Vision</x:v>
+        <x:v>Vision PC 동작</x:v>
       </x:c>
       <x:c r="F211" s="121" t="str">
-        <x:v>Prc Process COMPLETE</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="212" ht="70" customHeight="1">
+        <x:v>완료 기준 / 다음 단계</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="212" ht="165" customHeight="1">
       <x:c r="A212" s="20" t="str">
-        <x:v>ON</x:v>
+        <x:v>공통1</x:v>
       </x:c>
       <x:c r="B212" s="17" t="str">
-        <x:v>가공 중</x:v>
+        <x:v>측정 i 시퀀스 시작
+1900 1회</x:v>
       </x:c>
       <x:c r="C212" s="17" t="str">
-        <x:v>미완료</x:v>
-      </x:c>
-      <x:c r="D212" s="17" t="str">
-        <x:v>가공·0선 병행</x:v>
-      </x:c>
-      <x:c r="E212" s="17" t="str">
-        <x:v>현재 계획 수행</x:v>
-      </x:c>
-      <x:c r="F212" s="17" t="str">
-        <x:v>OFF</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="213" ht="90" customHeight="1">
+        <x:v>Stage Melsec 축 요청과 구분한다.</x:v>
+      </x:c>
+      <x:c r="D212" s="124" t="str">
+        <x:v>각 i=1~N의 IOF 전체 시퀀스 시작에서1900 요청/정상 응답을1회 확인한다. 이후 같은 시퀀스의1001→1002→1003 앞마다 다시 확인하지 않는다. 정상 N회면1900 요청 N회이며0선 OFF는 이 분기를 생략한다.</x:v>
+      </x:c>
+      <x:c r="E212" s="124" t="str">
+        <x:v>1900 요청/응답은 Cmd1900·UID0·Body0·Error0이다.1999는 별도 Heartbeat로 초기1900 응답을 대체하지 않는다.</x:v>
+      </x:c>
+      <x:c r="F212" s="124" t="str">
+        <x:v>성공 범위는 현재 Glass/i/연결 문맥이다. 이전 i의 성공을 다음 i의 초기 확인으로 재사용하지 않는다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="213" ht="165" customHeight="1">
       <x:c r="A213" s="20" t="str">
-        <x:v>ON</x:v>
+        <x:v>공통2</x:v>
       </x:c>
       <x:c r="B213" s="17" t="str">
-        <x:v>완료</x:v>
+        <x:v>초기1900 오류/불일치/Timeout</x:v>
       </x:c>
       <x:c r="C213" s="17" t="str">
-        <x:v>미완료</x:v>
-      </x:c>
-      <x:c r="D213" s="17" t="str">
-        <x:v>가공Done 보존 / 잔여0선 계속</x:v>
-      </x:c>
-      <x:c r="E213" s="17" t="str">
-        <x:v>촬영까지 유한 Y 주행 / TCP만 잔여면 정지 가능</x:v>
-      </x:c>
-      <x:c r="F213" s="17" t="str">
-        <x:v>OFF</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="214" ht="70" customHeight="1">
+        <x:v>이미 시작한 MOF와 Y 주행은 계속한다.</x:v>
+      </x:c>
+      <x:c r="D213" s="124" t="str">
+        <x:v>해당 i의1001/측정 후속을 시작하지 않고 원인·문맥·미완료를 남긴다.1002/1003 앞 추가1900으로 만회하는 흐름을 만들지 않는다.</x:v>
+      </x:c>
+      <x:c r="E213" s="124" t="str">
+        <x:v>잘못된 Cmd/UID/Len/Error 또는1999를 정상1900으로 취급하지 않는다.</x:v>
+      </x:c>
+      <x:c r="F213" s="124" t="str">
+        <x:v>정상 N회=N번과 오류/재시도 횟수는 구분한다. 복구·재시도 정책 수치는 계약으로 확정한다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="214" ht="180" customHeight="1">
       <x:c r="A214" s="20" t="str">
-        <x:v>ON</x:v>
+        <x:v>공통3</x:v>
       </x:c>
       <x:c r="B214" s="17" t="str">
-        <x:v>가공 중</x:v>
+        <x:v>연결 손실·늦은 응답
+새 시퀀스 경계</x:v>
       </x:c>
       <x:c r="C214" s="17" t="str">
-        <x:v>완료</x:v>
-      </x:c>
-      <x:c r="D214" s="17" t="str">
-        <x:v>0선Done 보존 / 가공 계속</x:v>
-      </x:c>
-      <x:c r="E214" s="17" t="str">
-        <x:v>현재 MOF 계속</x:v>
-      </x:c>
-      <x:c r="F214" s="17" t="str">
-        <x:v>OFF</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="215" ht="70" customHeight="1">
+        <x:v>1002 ACK 미수신 중에는 다음 X Request를 시작하지 않는다.</x:v>
+      </x:c>
+      <x:c r="D214" s="124" t="str">
+        <x:v>현재 거래·이미지/결과 문맥을 보존하고 연결 복구만으로 현재 시퀀스를 완료 처리하지 않는다. 새로운 시퀀스를 정식 시작하면 그 시작에서1900을1회 확인한다. 실패 세션·UID0 지연 응답 보호와 재동기화는 추가 설계다.</x:v>
+      </x:c>
+      <x:c r="E214" s="124" t="str">
+        <x:v>1002 상태 ACK와 검사 완료·1003 결과를 구분한다. 복구된 연결이 이전 버퍼 복구를 뜻하지 않는다.</x:v>
+      </x:c>
+      <x:c r="F214" s="124" t="str">
+        <x:v>현재 시퀀스 중간에1900을 임의로 재삽입하지 않는다. 재검/새 시퀀스 허용은 계약으로 확인한다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="215" ht="140" customHeight="1">
       <x:c r="A215" s="20" t="str">
-        <x:v>ON</x:v>
+        <x:v>공통4</x:v>
       </x:c>
       <x:c r="B215" s="17" t="str">
-        <x:v>완료</x:v>
+        <x:v>Process 도식의 화살표·방향 읽기</x:v>
       </x:c>
       <x:c r="C215" s="17" t="str">
-        <x:v>완료</x:v>
-      </x:c>
-      <x:c r="D215" s="17" t="str">
-        <x:v>두 시퀀스 합류 후 완료</x:v>
-      </x:c>
-      <x:c r="E215" s="17" t="str">
-        <x:v>Stage 실제 Y 종료는 별도 확인</x:v>
-      </x:c>
-      <x:c r="F215" s="17" t="str">
-        <x:v>ON</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="216" ht="70" customHeight="1">
-      <x:c r="A216" s="20" t="str">
-        <x:v>OFF</x:v>
-      </x:c>
-      <x:c r="B216" s="17" t="str">
-        <x:v>완료</x:v>
-      </x:c>
-      <x:c r="C216" s="17" t="str">
-        <x:v>해당없음</x:v>
-      </x:c>
-      <x:c r="D216" s="17" t="str">
-        <x:v>가공Done으로 완료</x:v>
-      </x:c>
-      <x:c r="E216" s="17" t="str">
-        <x:v>0선 좌표 읽기·ACS적용·측정 분기 없음</x:v>
-      </x:c>
-      <x:c r="F216" s="17" t="str">
-        <x:v>ON</x:v>
-      </x:c>
+        <x:v>남색 실선: Stage↔Process의 Melsec 신호/좌표/축 요청·완료.</x:v>
+      </x:c>
+      <x:c r="D215" s="124" t="str">
+        <x:v>주황 실선: Process→Vision TCP 요청. 초록 실선: Vision→Process TCP 응답/ACK/결과. 수평 화살촉이 수신자다.</x:v>
+      </x:c>
+      <x:c r="E215" s="124" t="str">
+        <x:v>보라 실선: Stage→Vision HW Trigger. Process Trigger 관측은 내부 동작 상자로 표시하고 미정 통신 경로를 만들지 않는다.</x:v>
+      </x:c>
+      <x:c r="F215" s="124" t="str">
+        <x:v>Process 도식의 세로선은 PC별 시간 흐름이며 메시지가 아니다. ACK 이후 X 이동과1003은 병행 경로다. 화살표 높이는 정확한 경과시간이나 양쪽 완료 시각 일치를 뜻하지 않는다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="216" ht="24" customHeight="1">
+      <x:c r="A216" s="3"/>
+      <x:c r="B216" s="3"/>
+      <x:c r="C216" s="3"/>
+      <x:c r="D216" s="3"/>
+      <x:c r="E216" s="3"/>
+      <x:c r="F216" s="3"/>
     </x:row>
     <x:row r="217" ht="24" customHeight="1">
       <x:c r="A217" s="3"/>
@@ -12632,89 +12560,145 @@
       <x:c r="E218" s="3"/>
       <x:c r="F218" s="3"/>
     </x:row>
-    <x:row r="219" ht="24" customHeight="1">
-      <x:c r="A219" s="7" t="str">
-        <x:v>1900 확인 범위</x:v>
-      </x:c>
-      <x:c r="B219" s="6"/>
-      <x:c r="C219" s="6"/>
-      <x:c r="D219" s="6"/>
-      <x:c r="E219" s="6"/>
-      <x:c r="F219" s="6"/>
-    </x:row>
-    <x:row r="220" ht="24" customHeight="1">
-      <x:c r="A220" s="125" t="str">
-        <x:v>0선 IOF 측정 i=1~N 각각의 시퀀스 시작에서1900 1회 확인 →1001 → LINE 촬영 →1002 ACK →1003 결과입니다. 정상 N회면1900 총 N번이며1002/1003 앞의 재확인은 없습니다.</x:v>
-      </x:c>
-      <x:c r="B220" s="6"/>
-      <x:c r="C220" s="6"/>
-      <x:c r="D220" s="6"/>
-      <x:c r="E220" s="6"/>
-      <x:c r="F220" s="6"/>
-    </x:row>
-    <x:row r="221" ht="24" customHeight="1">
-      <x:c r="A221" s="7" t="str">
-        <x:v>PEG 정보 기록 위치</x:v>
-      </x:c>
-      <x:c r="B221" s="6"/>
-      <x:c r="C221" s="6"/>
-      <x:c r="D221" s="6"/>
-      <x:c r="E221" s="6"/>
-      <x:c r="F221" s="6"/>
-    </x:row>
-    <x:row r="222" ht="24" customHeight="1">
-      <x:c r="A222" s="125" t="str">
-        <x:v>Process ABLE 조건 성립 + Process Ready 실제 위치 도착 확인 → PEG 정보 Melsec 게시 → Stage ACS 반영. Process Ready 위치 도착·정지 확인 후 Melsec에 PEG 위치 쓰기. 모든 PEG 정보는 이동 중 기록하지 않습니다.</x:v>
-      </x:c>
-      <x:c r="B222" s="6"/>
-      <x:c r="C222" s="6"/>
-      <x:c r="D222" s="6"/>
-      <x:c r="E222" s="6"/>
-      <x:c r="F222" s="6"/>
-    </x:row>
-    <x:row r="223" ht="24" customHeight="1">
-      <x:c r="A223" s="125" t="str">
-        <x:v>DoReady5에서는 PEG 내부 계획만 준비합니다. 현재 시나리오의 실제 PEG 위치 기록은 Process ABLE 조건과 Process Ready 도착 확인 후입니다. 0선 OFF면 Stage가0선 N/좌표를 읽거나 ACS에 적용하지 않고 이전0선 Trigger를 사용하지 않습니다.</x:v>
-      </x:c>
-      <x:c r="B223" s="6"/>
-      <x:c r="C223" s="6"/>
-      <x:c r="D223" s="6"/>
-      <x:c r="E223" s="6"/>
-      <x:c r="F223" s="6"/>
-    </x:row>
-    <x:row r="224" ht="24" customHeight="1">
-      <x:c r="A224" s="7" t="str">
-        <x:v>LINE 사이 병행과 시간 조건</x:v>
-      </x:c>
-      <x:c r="B224" s="6"/>
-      <x:c r="C224" s="6"/>
-      <x:c r="D224" s="6"/>
-      <x:c r="E224" s="6"/>
-      <x:c r="F224" s="6"/>
+    <x:row r="219" ht="32" customHeight="1">
+      <x:c r="A219" s="119" t="str">
+        <x:v>조건</x:v>
+      </x:c>
+      <x:c r="B219" s="120" t="str">
+        <x:v>실제 가공 상태</x:v>
+      </x:c>
+      <x:c r="C219" s="120" t="str">
+        <x:v>0선방어 상태</x:v>
+      </x:c>
+      <x:c r="D219" s="120" t="str">
+        <x:v>가공 SW 동작·데이터 업데이트</x:v>
+      </x:c>
+      <x:c r="E219" s="120" t="str">
+        <x:v>물리 주행 / Vision</x:v>
+      </x:c>
+      <x:c r="F219" s="121" t="str">
+        <x:v>Prc Process COMPLETE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="220" ht="70" customHeight="1">
+      <x:c r="A220" s="20" t="str">
+        <x:v>ON</x:v>
+      </x:c>
+      <x:c r="B220" s="17" t="str">
+        <x:v>가공 중</x:v>
+      </x:c>
+      <x:c r="C220" s="17" t="str">
+        <x:v>미완료</x:v>
+      </x:c>
+      <x:c r="D220" s="17" t="str">
+        <x:v>가공·0선 병행</x:v>
+      </x:c>
+      <x:c r="E220" s="17" t="str">
+        <x:v>현재 계획 수행</x:v>
+      </x:c>
+      <x:c r="F220" s="17" t="str">
+        <x:v>OFF</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="221" ht="90" customHeight="1">
+      <x:c r="A221" s="20" t="str">
+        <x:v>ON</x:v>
+      </x:c>
+      <x:c r="B221" s="17" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="C221" s="17" t="str">
+        <x:v>미완료</x:v>
+      </x:c>
+      <x:c r="D221" s="17" t="str">
+        <x:v>가공Done 보존 / 잔여0선 계속</x:v>
+      </x:c>
+      <x:c r="E221" s="17" t="str">
+        <x:v>촬영까지 유한 Y 주행 / TCP만 잔여면 정지 가능</x:v>
+      </x:c>
+      <x:c r="F221" s="17" t="str">
+        <x:v>OFF</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="222" ht="70" customHeight="1">
+      <x:c r="A222" s="20" t="str">
+        <x:v>ON</x:v>
+      </x:c>
+      <x:c r="B222" s="17" t="str">
+        <x:v>가공 중</x:v>
+      </x:c>
+      <x:c r="C222" s="17" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="D222" s="17" t="str">
+        <x:v>0선Done 보존 / 가공 계속</x:v>
+      </x:c>
+      <x:c r="E222" s="17" t="str">
+        <x:v>현재 MOF 계속</x:v>
+      </x:c>
+      <x:c r="F222" s="17" t="str">
+        <x:v>OFF</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="223" ht="70" customHeight="1">
+      <x:c r="A223" s="20" t="str">
+        <x:v>ON</x:v>
+      </x:c>
+      <x:c r="B223" s="17" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="C223" s="17" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="D223" s="17" t="str">
+        <x:v>두 시퀀스 합류 후 완료</x:v>
+      </x:c>
+      <x:c r="E223" s="17" t="str">
+        <x:v>Stage 실제 Y 종료는 별도 확인</x:v>
+      </x:c>
+      <x:c r="F223" s="17" t="str">
+        <x:v>ON</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="224" ht="70" customHeight="1">
+      <x:c r="A224" s="20" t="str">
+        <x:v>OFF</x:v>
+      </x:c>
+      <x:c r="B224" s="17" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="C224" s="17" t="str">
+        <x:v>해당없음</x:v>
+      </x:c>
+      <x:c r="D224" s="17" t="str">
+        <x:v>가공Done으로 완료</x:v>
+      </x:c>
+      <x:c r="E224" s="17" t="str">
+        <x:v>0선 좌표 읽기·ACS적용·측정 분기 없음</x:v>
+      </x:c>
+      <x:c r="F224" s="17" t="str">
+        <x:v>ON</x:v>
+      </x:c>
     </x:row>
     <x:row r="225" ht="24" customHeight="1">
-      <x:c r="A225" s="125" t="str">
-        <x:v>Process가 현재 i의1002 정상 ACK를 받은 뒤 다음 Review X(i+1)를 요청합니다. 마지막 노출 종료·X 허가·이전 요청 복귀도 확인합니다.1003 송신·응답·결과와는 독립으로 병행하며 ACK 전 다음 X 요청은 없습니다.</x:v>
-      </x:c>
-      <x:c r="B225" s="6"/>
-      <x:c r="C225" s="6"/>
-      <x:c r="D225" s="6"/>
-      <x:c r="E225" s="6"/>
-      <x:c r="F225" s="6"/>
+      <x:c r="A225" s="3"/>
+      <x:c r="B225" s="3"/>
+      <x:c r="C225" s="3"/>
+      <x:c r="D225" s="3"/>
+      <x:c r="E225" s="3"/>
+      <x:c r="F225" s="3"/>
     </x:row>
     <x:row r="226" ht="24" customHeight="1">
-      <x:c r="A226" s="125" t="str">
-        <x:v>다음 LINE 첫 Trigger 마감에는1002 ACK 수신 지연과 이후 X 이동·정착 시간을 포함합니다. 현재1003 결과→다음 시퀀스 초기1900/1001 경로는 별도로 검증합니다. Y 연속 주행과 오류 미완료 기준은 유지합니다.</x:v>
-      </x:c>
-      <x:c r="B226" s="6"/>
-      <x:c r="C226" s="6"/>
-      <x:c r="D226" s="6"/>
-      <x:c r="E226" s="6"/>
-      <x:c r="F226" s="6"/>
+      <x:c r="A226" s="3"/>
+      <x:c r="B226" s="3"/>
+      <x:c r="C226" s="3"/>
+      <x:c r="D226" s="3"/>
+      <x:c r="E226" s="3"/>
+      <x:c r="F226" s="3"/>
     </x:row>
     <x:row r="227" ht="24" customHeight="1">
       <x:c r="A227" s="7" t="str">
-        <x:v>검증할 데이터·피드백</x:v>
+        <x:v>1900 확인 범위</x:v>
       </x:c>
       <x:c r="B227" s="6"/>
       <x:c r="C227" s="6"/>
@@ -12724,7 +12708,7 @@
     </x:row>
     <x:row r="228" ht="24" customHeight="1">
       <x:c r="A228" s="125" t="str">
-        <x:v>Process Ready 수치/도착 피드백·오차, PEG 실제 주소/단위, LINE 시작/끝·실제 Trigger/노출/가공Done, Review X8011/8015/801B→8029와C124/C128의 범위/정착·복귀를 실제 계약과 대조합니다.</x:v>
+        <x:v>0선 IOF 측정 i=1~N 각각의 시퀀스 시작에서1900 1회 확인 →1001 → LINE 촬영 →1002 ACK →1003 결과입니다. 정상 N회면1900 총 N번이며1002/1003 앞의 재확인은 없습니다.</x:v>
       </x:c>
       <x:c r="B228" s="6"/>
       <x:c r="C228" s="6"/>
@@ -12733,8 +12717,8 @@
       <x:c r="F228" s="6"/>
     </x:row>
     <x:row r="229" ht="24" customHeight="1">
-      <x:c r="A229" s="125" t="str">
-        <x:v>1002 ACK는 검사 전체 완료가 아닙니다. LINE 측정 완료/1003 응답 준비 조건,1001/1003 길이·배열·실패 슬롯, 내부 Glass/LINE/Frame/업무 UID 대응은 Vision 계약으로 확인합니다. 미제공 완료 패킷을 임의로 만들지 않습니다.</x:v>
+      <x:c r="A229" s="7" t="str">
+        <x:v>PEG 정보 기록 위치</x:v>
       </x:c>
       <x:c r="B229" s="6"/>
       <x:c r="C229" s="6"/>
@@ -12744,7 +12728,7 @@
     </x:row>
     <x:row r="230" ht="24" customHeight="1">
       <x:c r="A230" s="125" t="str">
-        <x:v>최신 사용자 정정이 우선합니다. 이전 업무별1900 반복과1002 ACK 전 다음 X 선배치는 이번 개정으로 대체합니다. 첨부 IOF의 LINE별 준비·촬영·종료·결과와1002 ACK≠검사 완료는 유지합니다.</x:v>
+        <x:v>Process ABLE 조건 성립 + Process Ready 실제 위치 도착 확인 → PEG 정보 Melsec 게시 → Stage ACS 반영. Process Ready 위치 도착·정지 확인 후 Melsec에 PEG 위치 쓰기. 모든 PEG 정보는 이동 중 기록하지 않습니다.</x:v>
       </x:c>
       <x:c r="B230" s="6"/>
       <x:c r="C230" s="6"/>
@@ -12754,7 +12738,7 @@
     </x:row>
     <x:row r="231" ht="24" customHeight="1">
       <x:c r="A231" s="125" t="str">
-        <x:v>Process 도식의 화살표: 남색=Melsec(Stage↔Process), 주황=TCP 요청(Process→Vision), 초록=TCP 응답(Vision→Process), 보라=HW Trigger(Stage→Vision). 실선 화살촉이 수신자이며 세로선은 시간 흐름입니다.</x:v>
+        <x:v>DoReady5에서는 PEG 내부 계획만 준비합니다. 현재 시나리오의 실제 PEG 위치 기록은 Process ABLE 조건과 Process Ready 도착 확인 후입니다. 0선 OFF면 Stage가0선 N/좌표를 읽거나 ACS에 적용하지 않고 이전0선 Trigger를 사용하지 않습니다.</x:v>
       </x:c>
       <x:c r="B231" s="6"/>
       <x:c r="C231" s="6"/>
@@ -12763,8 +12747,8 @@
       <x:c r="F231" s="6"/>
     </x:row>
     <x:row r="232" ht="24" customHeight="1">
-      <x:c r="A232" s="125" t="str">
-        <x:v>가공Done·Y 주행Done·LINE 촬영Done·0선Done·상위 COMPLETE는 구분합니다. ON의 정상 완료는 가공Done AND0선Done, OFF는 가공Done입니다. 일반 측정/TCP 오류로 현재 MOF를 중도 정지하지 않습니다.</x:v>
+      <x:c r="A232" s="7" t="str">
+        <x:v>LINE 사이 병행과 시간 조건</x:v>
       </x:c>
       <x:c r="B232" s="6"/>
       <x:c r="C232" s="6"/>
@@ -12773,8 +12757,8 @@
       <x:c r="F232" s="6"/>
     </x:row>
     <x:row r="233" ht="24" customHeight="1">
-      <x:c r="A233" s="7" t="str">
-        <x:v>원본과 검증 범위</x:v>
+      <x:c r="A233" s="125" t="str">
+        <x:v>Process가 현재 i의1002 정상 ACK를 받은 뒤 다음 Review X(i+1)를 요청합니다. 마지막 노출 종료·X 허가·이전 요청 복귀도 확인합니다.1003 송신·응답·결과와는 독립으로 병행하며 ACK 전 다음 X 요청은 없습니다.</x:v>
       </x:c>
       <x:c r="B233" s="6"/>
       <x:c r="C233" s="6"/>
@@ -12784,7 +12768,7 @@
     </x:row>
     <x:row r="234" ht="24" customHeight="1">
       <x:c r="A234" s="125" t="str">
-        <x:v>최신 사용자 문구 수정·첨부 Auto/Manual IOF 도식, A3LD_Interface(Vision-Process).pptx 6/12/13장, Stage IF/MelsecMap Ver0.04, 읽기전용 MeasureVisionLine 흐름. 실제Melsec TODO/임시대기가 있어 생산 구현 완료 근거로 사용하지 않습니다.</x:v>
+        <x:v>다음 LINE 첫 Trigger 마감에는1002 ACK 수신 지연과 이후 X 이동·정착 시간을 포함합니다. 현재1003 결과→다음 시퀀스 초기1900/1001 경로는 별도로 검증합니다. Y 연속 주행과 오류 미완료 기준은 유지합니다.</x:v>
       </x:c>
       <x:c r="B234" s="6"/>
       <x:c r="C234" s="6"/>
@@ -12793,8 +12777,8 @@
       <x:c r="F234" s="6"/>
     </x:row>
     <x:row r="235" ht="24" customHeight="1">
-      <x:c r="A235" s="125" t="str">
-        <x:v>시나리오·평가 문서이며 실장비 통신/축/레이저 시험을 대신하지 않습니다. 구시뮬 전체Y종료를 실제 레이저 출사 종료로 해석하지 않습니다.</x:v>
+      <x:c r="A235" s="7" t="str">
+        <x:v>검증할 데이터·피드백</x:v>
       </x:c>
       <x:c r="B235" s="6"/>
       <x:c r="C235" s="6"/>
@@ -12803,48 +12787,128 @@
       <x:c r="F235" s="6"/>
     </x:row>
     <x:row r="236" ht="24" customHeight="1">
-      <x:c r="A236" s="3"/>
-      <x:c r="B236" s="3"/>
-      <x:c r="C236" s="3"/>
-      <x:c r="D236" s="3"/>
-      <x:c r="E236" s="3"/>
-      <x:c r="F236" s="3"/>
+      <x:c r="A236" s="125" t="str">
+        <x:v>Process Ready 수치/도착 피드백·오차, PEG 실제 주소/단위, LINE 시작/끝·실제 Trigger/노출/가공Done, Review X8011/8015/801B→8029와C124/C128의 범위/정착·복귀를 실제 계약과 대조합니다.</x:v>
+      </x:c>
+      <x:c r="B236" s="6"/>
+      <x:c r="C236" s="6"/>
+      <x:c r="D236" s="6"/>
+      <x:c r="E236" s="6"/>
+      <x:c r="F236" s="6"/>
     </x:row>
     <x:row r="237" ht="24" customHeight="1">
-      <x:c r="A237" s="3"/>
-      <x:c r="B237" s="3"/>
-      <x:c r="C237" s="3"/>
-      <x:c r="D237" s="3"/>
-      <x:c r="E237" s="3"/>
-      <x:c r="F237" s="3"/>
+      <x:c r="A237" s="125" t="str">
+        <x:v>1002 ACK는 검사 전체 완료가 아닙니다. LINE 측정 완료/1003 응답 준비 조건,1001/1003 길이·배열·실패 슬롯, 내부 Glass/LINE/Frame/업무 UID 대응은 Vision 계약으로 확인합니다. 미제공 완료 패킷을 임의로 만들지 않습니다.</x:v>
+      </x:c>
+      <x:c r="B237" s="6"/>
+      <x:c r="C237" s="6"/>
+      <x:c r="D237" s="6"/>
+      <x:c r="E237" s="6"/>
+      <x:c r="F237" s="6"/>
     </x:row>
     <x:row r="238" ht="24" customHeight="1">
-      <x:c r="A238" s="3"/>
-      <x:c r="B238" s="3"/>
-      <x:c r="C238" s="3"/>
-      <x:c r="D238" s="3"/>
-      <x:c r="E238" s="3"/>
-      <x:c r="F238" s="3"/>
+      <x:c r="A238" s="125" t="str">
+        <x:v>최신 사용자 정정이 우선합니다. 이전 업무별1900 반복과1002 ACK 전 다음 X 선배치는 이번 개정으로 대체합니다. 첨부 IOF의 LINE별 준비·촬영·종료·결과와1002 ACK≠검사 완료는 유지합니다.</x:v>
+      </x:c>
+      <x:c r="B238" s="6"/>
+      <x:c r="C238" s="6"/>
+      <x:c r="D238" s="6"/>
+      <x:c r="E238" s="6"/>
+      <x:c r="F238" s="6"/>
     </x:row>
     <x:row r="239" ht="24" customHeight="1">
-      <x:c r="A239" s="3"/>
-      <x:c r="B239" s="3"/>
-      <x:c r="C239" s="3"/>
-      <x:c r="D239" s="3"/>
-      <x:c r="E239" s="3"/>
-      <x:c r="F239" s="3"/>
+      <x:c r="A239" s="125" t="str">
+        <x:v>Process 도식의 화살표: 남색=Melsec(Stage↔Process), 주황=TCP 요청(Process→Vision), 초록=TCP 응답(Vision→Process), 보라=HW Trigger(Stage→Vision). 실선 화살촉이 수신자이며 세로선은 시간 흐름입니다.</x:v>
+      </x:c>
+      <x:c r="B239" s="6"/>
+      <x:c r="C239" s="6"/>
+      <x:c r="D239" s="6"/>
+      <x:c r="E239" s="6"/>
+      <x:c r="F239" s="6"/>
     </x:row>
     <x:row r="240" ht="24" customHeight="1">
-      <x:c r="A240" s="3"/>
-      <x:c r="B240" s="3"/>
-      <x:c r="C240" s="3"/>
-      <x:c r="D240" s="3"/>
-      <x:c r="E240" s="3"/>
-      <x:c r="F240" s="3"/>
+      <x:c r="A240" s="125" t="str">
+        <x:v>가공Done·Y 주행Done·LINE 촬영Done·0선Done·상위 COMPLETE는 구분합니다. ON의 정상 완료는 가공Done AND0선Done, OFF는 가공Done입니다. 일반 측정/TCP 오류로 현재 MOF를 중도 정지하지 않습니다.</x:v>
+      </x:c>
+      <x:c r="B240" s="6"/>
+      <x:c r="C240" s="6"/>
+      <x:c r="D240" s="6"/>
+      <x:c r="E240" s="6"/>
+      <x:c r="F240" s="6"/>
+    </x:row>
+    <x:row r="241" ht="24" customHeight="1">
+      <x:c r="A241" s="7" t="str">
+        <x:v>원본과 검증 범위</x:v>
+      </x:c>
+      <x:c r="B241" s="6"/>
+      <x:c r="C241" s="6"/>
+      <x:c r="D241" s="6"/>
+      <x:c r="E241" s="6"/>
+      <x:c r="F241" s="6"/>
+    </x:row>
+    <x:row r="242" ht="24" customHeight="1">
+      <x:c r="A242" s="125" t="str">
+        <x:v>최신 사용자 문구 수정·첨부 Auto/Manual IOF 도식, A3LD_Interface(Vision-Process).pptx 6/12/13장, Stage IF/MelsecMap Ver0.04, 읽기전용 MeasureVisionLine 흐름. 실제Melsec TODO/임시대기가 있어 생산 구현 완료 근거로 사용하지 않습니다.</x:v>
+      </x:c>
+      <x:c r="B242" s="6"/>
+      <x:c r="C242" s="6"/>
+      <x:c r="D242" s="6"/>
+      <x:c r="E242" s="6"/>
+      <x:c r="F242" s="6"/>
+    </x:row>
+    <x:row r="243" ht="24" customHeight="1">
+      <x:c r="A243" s="125" t="str">
+        <x:v>시나리오·평가 문서이며 실장비 통신/축/레이저 시험을 대신하지 않습니다. 구시뮬 전체Y종료를 실제 레이저 출사 종료로 해석하지 않습니다.</x:v>
+      </x:c>
+      <x:c r="B243" s="6"/>
+      <x:c r="C243" s="6"/>
+      <x:c r="D243" s="6"/>
+      <x:c r="E243" s="6"/>
+      <x:c r="F243" s="6"/>
+    </x:row>
+    <x:row r="244" ht="24" customHeight="1">
+      <x:c r="A244" s="3"/>
+      <x:c r="B244" s="3"/>
+      <x:c r="C244" s="3"/>
+      <x:c r="D244" s="3"/>
+      <x:c r="E244" s="3"/>
+      <x:c r="F244" s="3"/>
+    </x:row>
+    <x:row r="245" ht="24" customHeight="1">
+      <x:c r="A245" s="3"/>
+      <x:c r="B245" s="3"/>
+      <x:c r="C245" s="3"/>
+      <x:c r="D245" s="3"/>
+      <x:c r="E245" s="3"/>
+      <x:c r="F245" s="3"/>
+    </x:row>
+    <x:row r="246" ht="24" customHeight="1">
+      <x:c r="A246" s="3"/>
+      <x:c r="B246" s="3"/>
+      <x:c r="C246" s="3"/>
+      <x:c r="D246" s="3"/>
+      <x:c r="E246" s="3"/>
+      <x:c r="F246" s="3"/>
+    </x:row>
+    <x:row r="247" ht="24" customHeight="1">
+      <x:c r="A247" s="3"/>
+      <x:c r="B247" s="3"/>
+      <x:c r="C247" s="3"/>
+      <x:c r="D247" s="3"/>
+      <x:c r="E247" s="3"/>
+      <x:c r="F247" s="3"/>
+    </x:row>
+    <x:row r="248" ht="24" customHeight="1">
+      <x:c r="A248" s="3"/>
+      <x:c r="B248" s="3"/>
+      <x:c r="C248" s="3"/>
+      <x:c r="D248" s="3"/>
+      <x:c r="E248" s="3"/>
+      <x:c r="F248" s="3"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing r:id="Rccdcecc5c95a4841"/>
+  <x:drawing r:id="Ra05af131c78d49a9"/>
 </x:worksheet>
 </file>
 

</xml_diff>